<commit_message>
Updated the Emergency Stop test with correct data
</commit_message>
<xml_diff>
--- a/test/Emergency_Stop_Test.xlsx
+++ b/test/Emergency_Stop_Test.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10503"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rasmuslykke/Documents/UNI/2. Semester/P2/Test_Excel/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rasmuslykke/Desktop/P2_Battery_Disassembly/test/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BA816362-1A52-F14C-A738-960CF641B97C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67CC9E7D-DF56-B340-8D5D-97557376560F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" xr2:uid="{D2250453-5E7A-8A47-8C0E-36E0F327490B}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16980" xr2:uid="{D2250453-5E7A-8A47-8C0E-36E0F327490B}"/>
   </bookViews>
   <sheets>
     <sheet name="Ark1" sheetId="1" r:id="rId1"/>
@@ -39,24 +39,39 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="5">
   <si>
-    <t>Time</t>
+    <t>Emergency Stop Test</t>
   </si>
   <si>
-    <t>Emergency Stop Test</t>
+    <t>Time (s)</t>
+  </si>
+  <si>
+    <t>Sucess</t>
+  </si>
+  <si>
+    <t>Fail</t>
+  </si>
+  <si>
+    <t>✓</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -80,8 +95,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -416,43 +432,79 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5AE04398-FCC2-1046-9DB2-FFE2A05B406D}">
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="19.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="B1" t="s">
-        <v>0</v>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>1</v>
       </c>
+      <c r="B2">
+        <v>0.35</v>
+      </c>
+      <c r="C2" t="s">
+        <v>4</v>
+      </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>2</v>
       </c>
+      <c r="B3">
+        <v>0.49</v>
+      </c>
+      <c r="C3" t="s">
+        <v>4</v>
+      </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>3</v>
       </c>
+      <c r="B4">
+        <v>0.41</v>
+      </c>
+      <c r="C4" t="s">
+        <v>4</v>
+      </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>4</v>
       </c>
+      <c r="B5">
+        <v>0.4</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>4</v>
+      </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>5</v>
+      </c>
+      <c r="B6">
+        <v>0.34</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>